<commit_message>
Progress so far on the qmd
Most things still need description, graphs about the data also needed
</commit_message>
<xml_diff>
--- a/outputs/cv_results.xlsx
+++ b/outputs/cv_results.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="k_8" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="k_8" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -654,58 +654,58 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1342</v>
+        <v>0.1442</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6817</v>
+        <v>0.6888</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7544999999999999</v>
+        <v>0.7756999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2099</v>
+        <v>0.1931</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8584000000000001</v>
+        <v>0.8685</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5945</v>
+        <v>0.5921</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5722</v>
+        <v>0.5715</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4094</v>
+        <v>0.4099</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7563</v>
+        <v>0.7558</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1228</v>
+        <v>0.1384</v>
       </c>
       <c r="L4" t="n">
-        <v>0.119</v>
+        <v>0.1321</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2505</v>
+        <v>0.281</v>
       </c>
       <c r="N4" t="n">
-        <v>0.0883</v>
+        <v>0.1067</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1418</v>
+        <v>0.1564</v>
       </c>
       <c r="P4" t="n">
-        <v>0.0139</v>
+        <v>0.0138</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0223</v>
+        <v>0.0221</v>
       </c>
       <c r="R4" t="n">
-        <v>0.0167</v>
+        <v>0.0215</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0147</v>
+        <v>0.0148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>